<commit_message>
adjust excel and app code
</commit_message>
<xml_diff>
--- a/RocketPy_26/TEMPLATE_SIM/TEMPLATE_SIM.xlsx
+++ b/RocketPy_26/TEMPLATE_SIM/TEMPLATE_SIM.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bcb4f73bfa3edb7b/Bureau/EPFL/ERT/Programmation/RocketPy/2026_C_FD_SIM_Rocketpy/Up_to_date/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/085522fb5f488138/Documents/GitHub/2026_C_FD_SIM_Rocketpy/RocketPy_26/TEMPLATE_SIM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="11_C9DD2F4FA7B08B6997265DCA874B396EB9AE37AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D8EA4219-98A1-4C16-B3EB-76FB9987DF04}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="11_C9DD2F4FA7B08B6997265DCA874B396EB9AE37AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3099110C-52F7-4525-A230-1F96ACEF57D4}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="197">
   <si>
     <t>Name</t>
   </si>
@@ -497,24 +497,12 @@
     <t>Eth non-consommé</t>
   </si>
   <si>
-    <t>m_eth_density</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Masse volumique eth </t>
-  </si>
-  <si>
     <t>m_lox_unused</t>
   </si>
   <si>
     <t xml:space="preserve">Lox non-consommé </t>
   </si>
   <si>
-    <t>m_lox_density</t>
-  </si>
-  <si>
-    <t>Masse volumique lox</t>
-  </si>
-  <si>
     <t>m_n2</t>
   </si>
   <si>
@@ -615,6 +603,30 @@
   </si>
   <si>
     <t>Static margin liftoff [c]</t>
+  </si>
+  <si>
+    <t>eth_temperature</t>
+  </si>
+  <si>
+    <t>Température en K</t>
+  </si>
+  <si>
+    <t>eth_pressure</t>
+  </si>
+  <si>
+    <t>Pression en Pa</t>
+  </si>
+  <si>
+    <t>eth_massic_frac</t>
+  </si>
+  <si>
+    <t>Fraction massique de l'eth dans le fuel (par rapport à l'eau)</t>
+  </si>
+  <si>
+    <t>lox_temperature</t>
+  </si>
+  <si>
+    <t>lox_pressure</t>
   </si>
 </sst>
 </file>
@@ -751,7 +763,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -770,10 +782,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -781,7 +789,12 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1105,11 +1118,11 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
       <c r="E2" s="9" t="s">
         <v>48</v>
       </c>
@@ -1165,11 +1178,11 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -1227,11 +1240,11 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="14" t="s">
+      <c r="A12" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -1256,11 +1269,11 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="14" t="s">
+      <c r="A15" s="12" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -1285,11 +1298,11 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="14" t="s">
+      <c r="A18" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="15"/>
-      <c r="C18" s="15"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
@@ -1336,11 +1349,11 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -1365,11 +1378,11 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="14" t="s">
+      <c r="A26" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
@@ -1394,11 +1407,11 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="14" t="s">
+      <c r="A29" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -1423,11 +1436,11 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="14" t="s">
+      <c r="A32" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="B32" s="15"/>
-      <c r="C32" s="15"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -1452,11 +1465,11 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="14" t="s">
+      <c r="A35" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -1514,11 +1527,11 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="14" t="s">
+      <c r="A41" s="12" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15"/>
+      <c r="B41" s="13"/>
+      <c r="C41" s="13"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -1543,11 +1556,11 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="14" t="s">
+      <c r="A44" s="12" t="s">
         <v>108</v>
       </c>
-      <c r="B44" s="15"/>
-      <c r="C44" s="15"/>
+      <c r="B44" s="13"/>
+      <c r="C44" s="13"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -1583,11 +1596,11 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="14" t="s">
+      <c r="A48" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="B48" s="15"/>
-      <c r="C48" s="15"/>
+      <c r="B48" s="13"/>
+      <c r="C48" s="13"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -1612,11 +1625,11 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="14" t="s">
+      <c r="A51" s="12" t="s">
         <v>118</v>
       </c>
-      <c r="B51" s="15"/>
-      <c r="C51" s="15"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="13"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -1696,11 +1709,11 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="14" t="s">
+      <c r="A59" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="B59" s="15"/>
-      <c r="C59" s="15"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="13"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
@@ -1732,6 +1745,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A15:C15"/>
@@ -1739,13 +1758,7 @@
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A44:C44"/>
     <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A12:C12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1754,7 +1767,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:C33"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="32" customWidth="1"/>
@@ -1774,11 +1787,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="14" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1815,11 +1828,11 @@
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="14" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1862,11 +1875,11 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="16" t="s">
+      <c r="A13" s="14" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1890,159 +1903,192 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>153</v>
+        <v>189</v>
       </c>
       <c r="B16">
-        <v>810</v>
+        <v>293.14999999999998</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>154</v>
+        <v>190</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>155</v>
-      </c>
-      <c r="B17">
-        <v>0.57699999999999996</v>
+        <v>191</v>
+      </c>
+      <c r="B17" s="18">
+        <v>6000000</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>156</v>
+        <v>192</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>157</v>
+        <v>193</v>
       </c>
       <c r="B18">
-        <v>1154</v>
+        <v>0.9</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B19">
-        <v>2.605</v>
+        <v>0.57699999999999996</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="16" t="s">
-        <v>161</v>
-      </c>
-      <c r="B20" s="13"/>
-      <c r="C20" s="13"/>
+      <c r="A20" t="s">
+        <v>195</v>
+      </c>
+      <c r="B20">
+        <v>90.15</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>190</v>
+      </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>162</v>
-      </c>
-      <c r="B21">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="B21" s="18">
+        <v>6000000</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="B22">
-        <v>0.2</v>
+        <v>2.605</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>164</v>
-      </c>
-      <c r="B23">
-        <v>0</v>
-      </c>
+      <c r="A23" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="B23" s="15"/>
+      <c r="C23" s="15"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="B24">
-        <v>0.123</v>
+        <v>300</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="B25">
-        <v>0</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B26">
-        <v>0.17499999999999999</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="B27" s="13"/>
-      <c r="C27" s="13"/>
+      <c r="A27" t="s">
+        <v>161</v>
+      </c>
+      <c r="B27">
+        <v>0.123</v>
+      </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B28">
         <v>0</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>170</v>
-      </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
       <c r="B29">
-        <v>3300</v>
-      </c>
-      <c r="C29" s="2" t="s">
-        <v>172</v>
-      </c>
+        <v>0.17499999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="B30" s="15"/>
+      <c r="C30" s="15"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>173</v>
+        <v>165</v>
+      </c>
+      <c r="B31">
+        <v>0</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>174</v>
-      </c>
-      <c r="B32" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>176</v>
-      </c>
-      <c r="B33">
+        <v>167</v>
+      </c>
+      <c r="B32">
+        <v>3300</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>170</v>
+      </c>
+      <c r="B35" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>172</v>
+      </c>
+      <c r="B36">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="5">
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A30:C30"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A2:C2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2072,11 +2118,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -2123,11 +2169,11 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="16" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2203,11 +2249,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -2365,13 +2411,13 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="17" t="s">
-        <v>177</v>
-      </c>
-      <c r="B2" s="15"/>
+        <v>173</v>
+      </c>
+      <c r="B2" s="13"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B3" s="7">
         <v>5500</v>
@@ -2379,7 +2425,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="11" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B4" s="7">
         <v>40411.022698499997</v>
@@ -2387,13 +2433,13 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
-        <v>180</v>
-      </c>
-      <c r="B5" s="15"/>
+        <v>176</v>
+      </c>
+      <c r="B5" s="13"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B6" s="7">
         <v>3807.5145338293319</v>
@@ -2401,7 +2447,7 @@
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="11" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B7" s="7">
         <v>3911.5145338293319</v>
@@ -2409,7 +2455,7 @@
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B8" s="7">
         <v>272.83375364988592</v>
@@ -2417,7 +2463,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B9" s="7">
         <v>66.099687856506478</v>
@@ -2425,7 +2471,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B10" s="7">
         <v>0.81504806695996479</v>
@@ -2433,7 +2479,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B11" s="7">
         <v>30.49613725715653</v>
@@ -2441,7 +2487,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="11" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B12" s="7">
         <v>165.6653175932592</v>
@@ -2449,13 +2495,13 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A13" s="17" t="s">
-        <v>188</v>
-      </c>
-      <c r="B13" s="15"/>
+        <v>184</v>
+      </c>
+      <c r="B13" s="13"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B14" s="7">
         <v>27.919218121086761</v>
@@ -2463,7 +2509,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A15" s="11" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B15" s="7">
         <v>3.3476788497937262</v>
@@ -2471,13 +2517,13 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A16" s="17" t="s">
-        <v>191</v>
-      </c>
-      <c r="B16" s="15"/>
+        <v>187</v>
+      </c>
+      <c r="B16" s="13"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B17" s="7">
         <v>3.3255509324656729</v>

</xml_diff>

<commit_message>
add an inertial mode and tests
</commit_message>
<xml_diff>
--- a/RocketPy_26/TEMPLATE_SIM/TEMPLATE_SIM.xlsx
+++ b/RocketPy_26/TEMPLATE_SIM/TEMPLATE_SIM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/085522fb5f488138/Documents/GitHub/2026_C_FD_SIM_Rocketpy/RocketPy_26/TEMPLATE_SIM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="32" documentId="11_C9DD2F4FA7B08B6997265DCA874B396EB9AE37AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3099110C-52F7-4525-A230-1F96ACEF57D4}"/>
+  <xr:revisionPtr revIDLastSave="34" documentId="11_C9DD2F4FA7B08B6997265DCA874B396EB9AE37AC" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A5871062-E538-45E9-8916-35A9B14CF605}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Structure" sheetId="1" r:id="rId1"/>
@@ -782,19 +782,19 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="165" fontId="5" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -810,6 +810,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1118,11 +1122,11 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
       <c r="E2" s="9" t="s">
         <v>48</v>
       </c>
@@ -1178,11 +1182,11 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
@@ -1240,11 +1244,11 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="12" t="s">
+      <c r="A12" s="15" t="s">
         <v>68</v>
       </c>
-      <c r="B12" s="13"/>
-      <c r="C12" s="13"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
@@ -1269,11 +1273,11 @@
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="12" t="s">
+      <c r="A15" s="15" t="s">
         <v>71</v>
       </c>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
@@ -1298,11 +1302,11 @@
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="12" t="s">
+      <c r="A18" s="15" t="s">
         <v>75</v>
       </c>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
@@ -1349,11 +1353,11 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="15" t="s">
         <v>82</v>
       </c>
-      <c r="B23" s="13"/>
-      <c r="C23" s="13"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -1378,11 +1382,11 @@
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="B26" s="13"/>
-      <c r="C26" s="13"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16"/>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
@@ -1407,11 +1411,11 @@
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="15" t="s">
         <v>88</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16"/>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
@@ -1436,11 +1440,11 @@
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="12" t="s">
+      <c r="A32" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="B32" s="13"/>
-      <c r="C32" s="13"/>
+      <c r="B32" s="16"/>
+      <c r="C32" s="16"/>
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
@@ -1465,11 +1469,11 @@
       </c>
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="12" t="s">
+      <c r="A35" s="15" t="s">
         <v>94</v>
       </c>
-      <c r="B35" s="13"/>
-      <c r="C35" s="13"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16"/>
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
@@ -1527,11 +1531,11 @@
       </c>
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="12" t="s">
+      <c r="A41" s="15" t="s">
         <v>104</v>
       </c>
-      <c r="B41" s="13"/>
-      <c r="C41" s="13"/>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16"/>
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
@@ -1556,11 +1560,11 @@
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="12" t="s">
+      <c r="A44" s="15" t="s">
         <v>108</v>
       </c>
-      <c r="B44" s="13"/>
-      <c r="C44" s="13"/>
+      <c r="B44" s="16"/>
+      <c r="C44" s="16"/>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
@@ -1596,11 +1600,11 @@
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="12" t="s">
+      <c r="A48" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="B48" s="13"/>
-      <c r="C48" s="13"/>
+      <c r="B48" s="16"/>
+      <c r="C48" s="16"/>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
@@ -1625,11 +1629,11 @@
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="12" t="s">
+      <c r="A51" s="15" t="s">
         <v>118</v>
       </c>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
+      <c r="B51" s="16"/>
+      <c r="C51" s="16"/>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
@@ -1709,11 +1713,11 @@
       </c>
     </row>
     <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="12" t="s">
+      <c r="A59" s="15" t="s">
         <v>133</v>
       </c>
-      <c r="B59" s="13"/>
-      <c r="C59" s="13"/>
+      <c r="B59" s="16"/>
+      <c r="C59" s="16"/>
     </row>
     <row r="60" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
@@ -1745,12 +1749,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="A59:C59"/>
-    <mergeCell ref="A48:C48"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A41:C41"/>
-    <mergeCell ref="A44:C44"/>
-    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A51:C51"/>
     <mergeCell ref="A15:C15"/>
@@ -1760,6 +1758,12 @@
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A23:C23"/>
     <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A59:C59"/>
+    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A41:C41"/>
+    <mergeCell ref="A44:C44"/>
+    <mergeCell ref="A32:C32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1787,11 +1791,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="14" t="s">
+      <c r="A2" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -1828,11 +1832,11 @@
       <c r="C6" s="2"/>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="13" t="s">
         <v>143</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -1875,11 +1879,11 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="14" t="s">
+      <c r="A13" s="13" t="s">
         <v>149</v>
       </c>
-      <c r="B13" s="15"/>
-      <c r="C13" s="15"/>
+      <c r="B13" s="14"/>
+      <c r="C13" s="14"/>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
@@ -1916,7 +1920,7 @@
       <c r="A17" t="s">
         <v>191</v>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="12">
         <v>6000000</v>
       </c>
       <c r="C17" s="2" t="s">
@@ -1960,7 +1964,7 @@
       <c r="A21" t="s">
         <v>196</v>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="12">
         <v>6000000</v>
       </c>
       <c r="C21" s="2" t="s">
@@ -1979,11 +1983,11 @@
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="14" t="s">
+      <c r="A23" s="13" t="s">
         <v>157</v>
       </c>
-      <c r="B23" s="15"/>
-      <c r="C23" s="15"/>
+      <c r="B23" s="14"/>
+      <c r="C23" s="14"/>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
@@ -2034,11 +2038,11 @@
       </c>
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="13" t="s">
         <v>164</v>
       </c>
-      <c r="B30" s="15"/>
-      <c r="C30" s="15"/>
+      <c r="B30" s="14"/>
+      <c r="C30" s="14"/>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
@@ -2118,11 +2122,11 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
+      <c r="B2" s="14"/>
+      <c r="C2" s="14"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
@@ -2169,11 +2173,11 @@
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A7" s="16" t="s">
+      <c r="A7" s="17" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15"/>
+      <c r="B7" s="14"/>
+      <c r="C7" s="14"/>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
@@ -2249,11 +2253,11 @@
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A16" s="16" t="s">
+      <c r="A16" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
+      <c r="B16" s="14"/>
+      <c r="C16" s="14"/>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
@@ -2410,10 +2414,10 @@
       <c r="B1" s="7"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="B2" s="13"/>
+      <c r="B2" s="16"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
@@ -2432,10 +2436,10 @@
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A5" s="17" t="s">
+      <c r="A5" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="B5" s="13"/>
+      <c r="B5" s="16"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="11" t="s">
@@ -2494,10 +2498,10 @@
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B13" s="13"/>
+      <c r="B13" s="16"/>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A14" s="11" t="s">
@@ -2516,10 +2520,10 @@
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="16"/>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">

</xml_diff>